<commit_message>
Tableau synthese: enlever 'Djibril' du nom (AHMED MOUSSA Said)
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assets/files/tableau-synthese-e5.xlsx
+++ b/assets/files/tableau-synthese-e5.xlsx
@@ -1213,7 +1213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ35"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="12.75"/>
   <cols>
     <col width="70.42578125" customWidth="1" style="1" min="1" max="1"/>
@@ -1245,7 +1245,7 @@
     <row r="3" ht="39.95" customHeight="1">
       <c r="A3" s="48" t="inlineStr">
         <is>
-          <t>NOM et prénom : AHMED MOUSSA Saïd-Djibril</t>
+          <t>NOM et prénom : AHMED MOUSSA Saïd</t>
         </is>
       </c>
       <c r="B3" s="49" t="n"/>
@@ -1902,52 +1902,6 @@
       <c r="G35" s="4" t="n"/>
       <c r="H35" s="4" t="n"/>
     </row>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="A4:E4"/>

</xml_diff>

<commit_message>
feat(e5): remplir tableau synthese officiel + PDF + ajout GLPI competences
- Remplit l'Excel officiel BTS SIO 2026 (Annexe VI-1) avec les 9 realisations
  Formation : ClassCord, Wiki Outline, Windows Server, Parc AD, Supervision,
  Infra IRIS, GLPI SISR+SLAM
  1ere annee pro : Alternance Kine@dom
  2eme annee pro : Smart Projector IRIS
- Exporte en PDF via Excel COM (178 KB, format A3 paysage officiel)
- Ajoute GLPI comme projet dans les competences BTS SIO :
  B1.1 Gerer le patrimoine (GLPI ITSM)
  B1.2 Mettre a disposition un service (GLPI)
  B1.3 Repondre aux incidents (GLPI Helpdesk)
  B2.2 Installer et deployer (GLPI Railway)

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assets/files/tableau-synthese-e5.xlsx
+++ b/assets/files/tableau-synthese-e5.xlsx
@@ -83,9 +83,12 @@
       <sz val="16"/>
     </font>
     <font>
-      <sz val="9"/>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
@@ -98,7 +101,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="42">
+  <borders count="41">
     <border>
       <left/>
       <right/>
@@ -615,27 +618,13 @@
       </top>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="00000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="00000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00000000"/>
-      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -802,14 +791,17 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1213,7 +1205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M35"/>
+  <dimension ref="A1:AQ35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="12.75"/>
   <cols>
     <col width="70.42578125" customWidth="1" style="1" min="1" max="1"/>
@@ -1280,12 +1272,12 @@
       </c>
       <c r="G4" s="17" t="inlineStr">
         <is>
-          <t>☒ SISR</t>
+          <t>☑ SISR</t>
         </is>
       </c>
       <c r="H4" s="25" t="inlineStr">
         <is>
-          <t>▢ SLAM</t>
+          <t>☐ SLAM</t>
         </is>
       </c>
     </row>
@@ -1412,19 +1404,17 @@
       <c r="G8" s="49" t="n"/>
       <c r="H8" s="50" t="n"/>
     </row>
-    <row r="9" ht="70" customFormat="1" customHeight="1" s="2">
+    <row r="9" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A9" s="62" t="inlineStr">
         <is>
           <t>ClassCord Server
-Serveur de chat TCP multi-clients (Python, systemd, Docker, fail2ban, SQLite). 1ère année.
-GitHub : github.com/sdjbrl/classcord_djibril</t>
+Déploiement serveur de chat TCP multi-clients : Python, systemd, Docker, fail2ban, SQLite.</t>
         </is>
       </c>
       <c r="B9" s="63" t="inlineStr">
         <is>
           <t>23/06/25
-au
-27/06/25</t>
+au 27/06/25</t>
         </is>
       </c>
       <c r="C9" s="64" t="inlineStr">
@@ -1437,7 +1427,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="E9" s="64" t="inlineStr"/>
+      <c r="E9" s="21" t="n"/>
       <c r="F9" s="64" t="inlineStr">
         <is>
           <t>X</t>
@@ -1448,21 +1438,19 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H9" s="64" t="inlineStr"/>
-    </row>
-    <row r="10" ht="70" customFormat="1" customHeight="1" s="2">
+      <c r="H9" s="22" t="n"/>
+    </row>
+    <row r="10" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A10" s="62" t="inlineStr">
         <is>
-          <t>Wiki Outline (binôme)
-Documentation collaborative : Docker Compose, PostgreSQL, Redis, MinIO, Traefik TLS, OIDC/Keycloak SSO.
-URL : wiki.iris.a3n.fr:4433 — GitHub : github.com/sdjbrl/wiki-iris</t>
+          <t>Wiki Outline
+Documentation collaborative Docker Compose : PostgreSQL, Redis, MinIO, Traefik TLS, OIDC/Keycloak.</t>
         </is>
       </c>
       <c r="B10" s="63" t="inlineStr">
         <is>
           <t>23/02/26
-au
-27/02/26</t>
+au 27/02/26</t>
         </is>
       </c>
       <c r="C10" s="64" t="inlineStr">
@@ -1470,7 +1458,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="D10" s="64" t="inlineStr"/>
+      <c r="D10" s="21" t="n"/>
       <c r="E10" s="64" t="inlineStr">
         <is>
           <t>X</t>
@@ -1486,25 +1474,23 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H10" s="64" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="70" customFormat="1" customHeight="1" s="2">
+      <c r="H10" s="65" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A11" s="62" t="inlineStr">
         <is>
-          <t>Windows Server 2022 — Vagrant
-Automatisation AD DS / DNS / DHCP / GPO / FSRM / WSUS / WDS via Vagrant et 10 scripts PowerShell idempotents.
-GitHub : github.com/Mediaschool-IRIS-BTS-SISR-2025/TP_WS_Said</t>
+          <t>Windows Server Vagrant
+Automatisation AD DS / DNS / DHCP / GPO / FSRM / WSUS / WDS via Vagrant et 10 scripts PowerShell.</t>
         </is>
       </c>
       <c r="B11" s="63" t="inlineStr">
         <is>
           <t>23/03/26
-au
-27/03/26</t>
+au 27/03/26</t>
         </is>
       </c>
       <c r="C11" s="64" t="inlineStr">
@@ -1512,8 +1498,8 @@
           <t>X</t>
         </is>
       </c>
-      <c r="D11" s="64" t="inlineStr"/>
-      <c r="E11" s="64" t="inlineStr"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
       <c r="F11" s="64" t="inlineStr">
         <is>
           <t>X</t>
@@ -1524,23 +1510,23 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H11" s="64" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="70" customFormat="1" customHeight="1" s="2">
+      <c r="H11" s="65" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A12" s="62" t="inlineStr">
         <is>
-          <t>Parc AD DS familial (projet personnel)
-Domaine Active Directory domestique, GPO par profil (parents/enfants), partages réseau, supervision PowerShell.</t>
+          <t>Parc AD DS familial
+Domaine Active Directory domestique, GPO par profil, partages réseau, supervision PowerShell.</t>
         </is>
       </c>
       <c r="B12" s="63" t="inlineStr">
         <is>
           <t>01/04/25
-en cours</t>
+— en cours</t>
         </is>
       </c>
       <c r="C12" s="64" t="inlineStr">
@@ -1548,8 +1534,8 @@
           <t>X</t>
         </is>
       </c>
-      <c r="D12" s="64" t="inlineStr"/>
-      <c r="E12" s="64" t="inlineStr"/>
+      <c r="D12" s="21" t="n"/>
+      <c r="E12" s="21" t="n"/>
       <c r="F12" s="64" t="inlineStr">
         <is>
           <t>X</t>
@@ -1560,20 +1546,19 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H12" s="64" t="inlineStr"/>
-    </row>
-    <row r="13" ht="70" customFormat="1" customHeight="1" s="2">
+      <c r="H12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A13" s="62" t="inlineStr">
         <is>
           <t>Supervision Serveur IRIS
-Stack Prometheus + Grafana + Node-Exporter + cAdvisor + Loki + Promtail. Benchmark de 4 solutions, dashboards, alerting Alertmanager.</t>
+Stack Prometheus + Grafana + Node-Exporter + cAdvisor + Loki + Promtail. Dashboards + alerting.</t>
         </is>
       </c>
       <c r="B13" s="63" t="inlineStr">
         <is>
           <t>23/02/26
-au
-27/02/26</t>
+au 27/02/26</t>
         </is>
       </c>
       <c r="C13" s="64" t="inlineStr">
@@ -1581,8 +1566,8 @@
           <t>X</t>
         </is>
       </c>
-      <c r="D13" s="64" t="inlineStr"/>
-      <c r="E13" s="64" t="inlineStr"/>
+      <c r="D13" s="21" t="n"/>
+      <c r="E13" s="21" t="n"/>
       <c r="F13" s="64" t="inlineStr">
         <is>
           <t>X</t>
@@ -1593,24 +1578,23 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H13" s="64" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="70" customFormat="1" customHeight="1" s="2">
+      <c r="H13" s="65" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A14" s="62" t="inlineStr">
         <is>
-          <t>Infrastructure Réseau &amp; Virtualisation IRIS — PROP-IRIS-v4 (binôme)
-5 VLANs, 802.1X / FreeRADIUS / OpenLDAP, KVM natif + 60 VMs SISR (WS2022 / Debian), Docker SLAM + Dockhand, BorgBackup.</t>
+          <t>Infrastructure Réseau &amp; Virtualisation IRIS (PROP-IRIS-v4)
+5 VLANs, 802.1X/FreeRADIUS/OpenLDAP, KVM + 60 VMs, Docker SLAM, BorgBackup.</t>
         </is>
       </c>
       <c r="B14" s="63" t="inlineStr">
         <is>
           <t>24/02/26
-au
-28/02/26</t>
+au 28/02/26</t>
         </is>
       </c>
       <c r="C14" s="64" t="inlineStr">
@@ -1618,8 +1602,8 @@
           <t>X</t>
         </is>
       </c>
-      <c r="D14" s="64" t="inlineStr"/>
-      <c r="E14" s="64" t="inlineStr"/>
+      <c r="D14" s="21" t="n"/>
+      <c r="E14" s="21" t="n"/>
       <c r="F14" s="64" t="inlineStr">
         <is>
           <t>X</t>
@@ -1630,21 +1614,50 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H14" s="64" t="inlineStr">
+      <c r="H14" s="65" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
     </row>
     <row r="15" ht="39.95" customFormat="1" customHeight="1" s="2">
-      <c r="A15" s="13" t="n"/>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="21" t="n"/>
-      <c r="D15" s="21" t="n"/>
+      <c r="A15" s="62" t="inlineStr">
+        <is>
+          <t>GLPI — ITSM conteneurisé (SISR + SLAM)
+GLPI 10.0.18, Apache 2.4 + PHP 8.2 + MariaDB, HTTPS Railway, domaine glpi.saiddev.fr, lab Vagrant.</t>
+        </is>
+      </c>
+      <c r="B15" s="63" t="inlineStr">
+        <is>
+          <t>23/04/26</t>
+        </is>
+      </c>
+      <c r="C15" s="64" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D15" s="64" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="E15" s="21" t="n"/>
-      <c r="F15" s="21" t="n"/>
-      <c r="G15" s="21" t="n"/>
-      <c r="H15" s="22" t="n"/>
+      <c r="F15" s="64" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G15" s="64" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H15" s="65" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A16" s="13" t="n"/>
@@ -1690,19 +1703,17 @@
       <c r="G19" s="54" t="n"/>
       <c r="H19" s="55" t="n"/>
     </row>
-    <row r="20" ht="70" customFormat="1" customHeight="1" s="2">
+    <row r="20" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A20" s="62" t="inlineStr">
         <is>
           <t>Alternance Kiné@dom Nice (Ephycient)
-Support helpdesk N1/N2 via ticketing interne (personnel administratif &amp; kinésithérapeutes), maintenance d'un parc de 15 postes, exploitation du SaaS métier Ephycient (planification tournées, dossiers patients, facturation), conformité RGPD santé. SLA informel &lt; 24 h.
-Fiche projet : sdjbrl.me/projects/kineadom.html</t>
+Support helpdesk N1/N2, maintenance parc 15 postes, exploitation SaaS Ephycient, conformité RGPD.</t>
         </is>
       </c>
       <c r="B20" s="63" t="inlineStr">
         <is>
           <t>16/09/24
-au
-18/07/25</t>
+au 18/07/25</t>
         </is>
       </c>
       <c r="C20" s="64" t="inlineStr">
@@ -1715,10 +1726,10 @@
           <t>X</t>
         </is>
       </c>
-      <c r="E20" s="64" t="inlineStr"/>
-      <c r="F20" s="64" t="inlineStr"/>
-      <c r="G20" s="64" t="inlineStr"/>
-      <c r="H20" s="64" t="inlineStr"/>
+      <c r="E20" s="21" t="n"/>
+      <c r="F20" s="21" t="n"/>
+      <c r="G20" s="21" t="n"/>
+      <c r="H20" s="22" t="n"/>
     </row>
     <row r="21" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A21" s="13" t="n"/>
@@ -1794,19 +1805,17 @@
       <c r="G27" s="54" t="n"/>
       <c r="H27" s="55" t="n"/>
     </row>
-    <row r="28" ht="70" customFormat="1" customHeight="1" s="2">
+    <row r="28" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A28" s="62" t="inlineStr">
         <is>
-          <t>Smart Projector IRIS — Stage SISR
-Automatisation des vidéoprojecteurs (10 salles) : Raspberry Pi 4 + relais GPIO + commutateur HDMI, interface web Flask. Pilote 2 salles puis rollout complet à IRIS Nice.
-Fiche projet : sdjbrl.me/projects/smart-projector.html</t>
+          <t>Smart Projector IRIS — Stage 2ᵉ année
+Automatisation vidéoprojecteurs 10 salles : Raspberry Pi 4, relais GPIO, HDMI, interface Flask.</t>
         </is>
       </c>
       <c r="B28" s="63" t="inlineStr">
         <is>
           <t>05/01/26
-au
-14/02/26</t>
+au 14/02/26</t>
         </is>
       </c>
       <c r="C28" s="64" t="inlineStr">
@@ -1819,7 +1828,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="E28" s="64" t="inlineStr"/>
+      <c r="E28" s="21" t="n"/>
       <c r="F28" s="64" t="inlineStr">
         <is>
           <t>X</t>
@@ -1830,7 +1839,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="H28" s="64" t="inlineStr"/>
+      <c r="H28" s="22" t="n"/>
     </row>
     <row r="29" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A29" s="13" t="n"/>
@@ -1902,6 +1911,52 @@
       <c r="G35" s="4" t="n"/>
       <c r="H35" s="4" t="n"/>
     </row>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="A4:E4"/>

</xml_diff>